<commit_message>
2 new funcrtions added GetRowAddress and GetLastRowAddress
</commit_message>
<xml_diff>
--- a/3-Dev/DevApp/Files/datatableHasEmptyRow.xlsx
+++ b/3-Dev/DevApp/Files/datatableHasEmptyRow.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a990f455bb745add/ProjetsDev/10-Pierlam/OpenExcelSdk/Dev/OpenExcelSdk/3-Dev/DevApp/Files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7" documentId="11_AD4DB114E441178AC67DF4536695FF58683EDF1B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D38BC85A-BFD5-44F6-93CA-28EDC54BA36D}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="11_AD4DB114E441178AC67DF4536695FF58683EDF1B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B0200EB8-46F3-454D-BF25-97B8843AE534}"/>
   <bookViews>
     <workbookView xWindow="9630" yWindow="2520" windowWidth="19125" windowHeight="10530" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -87,6 +87,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -352,7 +356,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -370,8 +374,8 @@
         <v>45</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6">
         <v>57</v>
       </c>
     </row>

</xml_diff>